<commit_message>
R17 mild -> strong
</commit_message>
<xml_diff>
--- a/test/4. HACKATHON_FRAML_RULES.xlsx
+++ b/test/4. HACKATHON_FRAML_RULES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://capgemini-my.sharepoint.com/personal/dorota_grzybowska_capgemini_com/Documents/Desktop/Szkolenia/HACKATHON Python 2025/DOKUMENTY/Final/FINAL _FINAL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source\Hakaton\fraudd\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8B648CB-BC91-4692-8EDF-AE3DF51C2AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B13B0AF-8982-4AC7-88AB-E32F3F3D1045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B3A44CC-A8E7-445D-811A-288200A6BF4C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{1B3A44CC-A8E7-445D-811A-288200A6BF4C}"/>
   </bookViews>
   <sheets>
     <sheet name="FRAML Rules" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="106">
   <si>
     <t>Rule ID</t>
   </si>
@@ -1262,7 +1262,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1843,7 +1843,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D39EB031-8D3A-4F37-8C82-0147BF841D49}">
   <dimension ref="A1:L15"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" style="18" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" style="1" customWidth="1"/>
@@ -1860,7 +1860,7 @@
     <col min="13" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="96" customHeight="1">
+    <row r="1" spans="1:12" ht="96" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="133.9" customHeight="1">
+    <row r="2" spans="1:12" ht="133.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>12</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="155.44999999999999" customHeight="1">
+    <row r="3" spans="1:12" ht="155.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>23</v>
       </c>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="L3" s="20"/>
     </row>
-    <row r="4" spans="1:12" ht="45">
+    <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
         <v>30</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="91.9" customHeight="1">
+    <row r="5" spans="1:12" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
         <v>36</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="45">
+    <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
         <v>45</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="75">
+    <row r="7" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>50</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="101.25" customHeight="1">
+    <row r="8" spans="1:12" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>56</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="105">
+    <row r="9" spans="1:12" ht="105" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>63</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="180">
+    <row r="10" spans="1:12" ht="180" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
         <v>69</v>
       </c>
@@ -2220,7 +2220,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="60">
+    <row r="11" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
         <v>75</v>
       </c>
@@ -2236,7 +2236,9 @@
       <c r="E11" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>17</v>
+      </c>
       <c r="G11" s="8">
         <v>15</v>
       </c>
@@ -2254,7 +2256,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="60">
+    <row r="12" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
         <v>82</v>
       </c>
@@ -2290,7 +2292,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="270">
+    <row r="13" spans="1:12" ht="270" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>88</v>
       </c>
@@ -2328,7 +2330,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>95</v>
       </c>
@@ -2362,7 +2364,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="75">
+    <row r="15" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>101</v>
       </c>
@@ -2413,15 +2415,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010045BF1A5D1A7DC7448263498994A172CC" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="80061a75a75cd06188a47c4ba574d57e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6aa2d33d-672c-4c5a-a9f5-a5d7220a9a33" xmlns:ns3="2316f3af-75b1-4ca8-829c-1fc88bf82c40" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="80766c03347fa849f777b73755204753" ns2:_="" ns3:_="">
     <xsd:import namespace="6aa2d33d-672c-4c5a-a9f5-a5d7220a9a33"/>
@@ -2628,16 +2621,49 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FA0EEB1-3F36-4145-8B71-3EA704840E7A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FA0EEB1-3F36-4145-8B71-3EA704840E7A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B213E9C-3D83-4259-95E7-9513CF648464}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1D8F09E-9ADD-487E-865D-7DDCBFD63892}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6aa2d33d-672c-4c5a-a9f5-a5d7220a9a33"/>
+    <ds:schemaRef ds:uri="2316f3af-75b1-4ca8-829c-1fc88bf82c40"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1D8F09E-9ADD-487E-865D-7DDCBFD63892}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B213E9C-3D83-4259-95E7-9513CF648464}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>